<commit_message>
added intended action as reqruied field for input
</commit_message>
<xml_diff>
--- a/preprocessorEC/data/upload_template.xlsx
+++ b/preprocessorEC/data/upload_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://montefioreorg-my.sharepoint.com/personal/dli2_montefiore_org/Documents/Documents/A8 - Contract Atlas/preprocessorEC/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dli2\OneDrive - Montefiore Medicine\Documents\A8 - Contract Atlas\preprocessorEC\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="11_4CE123EBF613C826CD1A4C73E4B3DB147452E70A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D0E93ED-DB61-4DCC-A646-8115549AD658}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B1C1F0E-086D-484A-A382-3FB70C0E0819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2610" yWindow="1980" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13365" yWindow="4635" windowWidth="28800" windowHeight="15150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="98">
   <si>
     <t>Mfg Part Num</t>
   </si>
@@ -321,6 +321,12 @@
   </si>
   <si>
     <t>Source Contract Type</t>
+  </si>
+  <si>
+    <t>Intended Action</t>
+  </si>
+  <si>
+    <t>Upsert</t>
   </si>
 </sst>
 </file>
@@ -706,7 +712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="55.28515625" customWidth="1"/>
@@ -715,7 +721,7 @@
     <col min="10" max="10" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -752,8 +758,11 @@
       <c r="L1" s="2" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -787,8 +796,11 @@
       <c r="L2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -822,8 +834,11 @@
       <c r="L3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -857,8 +872,11 @@
       <c r="L4" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -892,8 +910,11 @@
       <c r="L5" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -927,8 +948,11 @@
       <c r="L6" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -962,8 +986,11 @@
       <c r="L7" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -997,8 +1024,11 @@
       <c r="L8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1032,8 +1062,11 @@
       <c r="L9" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -1067,8 +1100,11 @@
       <c r="L10" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -1102,8 +1138,11 @@
       <c r="L11" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1137,8 +1176,11 @@
       <c r="L12" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -1172,8 +1214,11 @@
       <c r="L13" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -1207,8 +1252,11 @@
       <c r="L14" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M14" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1242,8 +1290,11 @@
       <c r="L15" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1277,8 +1328,11 @@
       <c r="L16" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M16" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1312,8 +1366,11 @@
       <c r="L17" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -1347,8 +1404,11 @@
       <c r="L18" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1382,8 +1442,11 @@
       <c r="L19" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1417,8 +1480,11 @@
       <c r="L20" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M20" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -1452,8 +1518,11 @@
       <c r="L21" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M21" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -1487,8 +1556,11 @@
       <c r="L22" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M22" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -1522,8 +1594,11 @@
       <c r="L23" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M23" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>57</v>
       </c>
@@ -1557,8 +1632,11 @@
       <c r="L24" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -1595,8 +1673,11 @@
       <c r="L25" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M25" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>59</v>
       </c>
@@ -1630,8 +1711,11 @@
       <c r="L26" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M26" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>60</v>
       </c>
@@ -1665,8 +1749,11 @@
       <c r="L27" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>61</v>
       </c>
@@ -1702,6 +1789,9 @@
       </c>
       <c r="L28" t="s">
         <v>71</v>
+      </c>
+      <c r="M28" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>